<commit_message>
Aligning with most recent Basic Plan for Electricity Supply and Demand
</commit_message>
<xml_diff>
--- a/InputData/elec/DRC/Demand Response Capacity.xlsx
+++ b/InputData/elec/DRC/Demand Response Capacity.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Dropbox\NEXT Group\90. 개인 폴더\이지우\단기대응\202501 EPS 수요전망\V3\DRC\old\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://energyinnovation.sharepoint.com/sites/ExternalSharing-PolicyExternal2/Shared Documents/Policy - Modeling and Analysis External/South Korea EPS/New Files_June/20260703/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01902E13-AAE6-4453-9394-D5CA716BD9DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="8_{90BDB88C-943A-44A0-9F6C-1B16932A1EDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1FC47F0E-F8C0-4B88-AADF-C883F16C7A19}"/>
   <bookViews>
-    <workbookView xWindow="2268" yWindow="2268" windowWidth="17280" windowHeight="8880" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-19305" yWindow="-4650" windowWidth="19410" windowHeight="20985" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="33">
   <si>
     <t>Year</t>
   </si>
@@ -84,9 +84,6 @@
   </si>
   <si>
     <t>Sources:</t>
-  </si>
-  <si>
-    <t>2019 Capacity and 2030 Projection</t>
   </si>
   <si>
     <t>MOTIE</t>
@@ -113,10 +110,6 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>BEFORE 2020 : same rate as 2021</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>Forecasted data</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
@@ -125,49 +118,61 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>AFTER 2034 : same rate as 2036</t>
+    <t>Unit: hours</t>
+  </si>
+  <si>
+    <t>DR Hours per DR Event</t>
+  </si>
+  <si>
+    <t>Hours per Event</t>
+  </si>
+  <si>
+    <t>DR Hours per Year and per Event</t>
+  </si>
+  <si>
+    <t>Hours of Shift DR per Year</t>
+  </si>
+  <si>
+    <t>Hours of DR per Event</t>
+  </si>
+  <si>
+    <t>Participants must be able to maintain demand reduction for at least 4 hours per DR event (전력거래소 등록시험 기준 3~4시간, 단 중소형 및 제주DR은 감축지속시간 1시간 적용)</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>10th basic electricity supply plan (2022~2036)</t>
+    <t>AFTER 2038 : same rate as 2038</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>https://new.kpx.or.kr/menu.es?mid=a10403070000</t>
+    <t>BEFORE 2024 : same rate as 2025</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>2022~2036: Data from 10th basic electricity supply plan</t>
+    <t>제11차 전력수급기본계획-3.수요관리목표-가.최대전력절감계획-DR시장(p.91)</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>2020, 2021: Incremental rate in 2022</t>
+    <t>2024 Capacity and 2038 Projection</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>2036~2050: Incremental rate in 2036</t>
+    <t>11th basic electricity supply plan (2024~2038)</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>Unit: hours</t>
-  </si>
-  <si>
-    <t>DR Hours per DR Event</t>
-  </si>
-  <si>
-    <t>Hours per Event</t>
-  </si>
-  <si>
-    <t>DR Hours per Year and per Event</t>
-  </si>
-  <si>
-    <t>Hours of Shift DR per Year</t>
-  </si>
-  <si>
-    <t>Hours of DR per Event</t>
-  </si>
-  <si>
-    <t>Participants must be able to maintain demand reduction for at least 4 hours per DR event (전력거래소 등록시험 기준 3~4시간, 단 중소형 및 제주DR은 감축지속시간 1시간 적용)</t>
+    <t>2024~2038: Data from 11th basic electricity supply plan</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>2038~2050: Incremental rate in 2038</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>2020~2023: Incremental rate in 2024</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.motir.go.kr/kor/article/ATCLc01b2801b/70152/view</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -175,11 +180,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -187,7 +192,7 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -195,13 +200,13 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="8"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -210,7 +215,7 @@
       <b/>
       <sz val="18"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -218,7 +223,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -227,7 +232,7 @@
       <b/>
       <sz val="14"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -235,7 +240,7 @@
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -243,7 +248,7 @@
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -251,12 +256,28 @@
       <i/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -281,13 +302,34 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBBBBBB"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBBBBBB"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBBBBBB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBBBBBB"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -321,11 +363,7 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
@@ -338,8 +376,6 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -348,10 +384,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="표준" xfId="0" builtinId="0"/>
-    <cellStyle name="하이퍼링크" xfId="1" builtinId="8"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -366,10 +406,59 @@
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>38101</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>44450</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>189558</xdr:colOff>
+      <xdr:row>54</xdr:row>
+      <xdr:rowOff>106376</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="그림 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F96F1D57-8CD9-836D-5AE6-62AD1A2F9EDB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="38101" y="4854575"/>
+          <a:ext cx="4809182" cy="7291401"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 테마">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -407,9 +496,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -442,26 +531,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -494,26 +566,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -687,98 +742,98 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B27"/>
-  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="28.59765625" customWidth="1"/>
+    <col min="2" max="2" width="28.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:2">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B4" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="B5" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="B5" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="B6" s="24">
-        <v>2022</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="B7" s="24" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="B8" s="15" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A11" s="1" t="s">
+    <row r="6" spans="1:2">
+      <c r="B6" s="20">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="B7" s="20" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="B8" s="27" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:2">
+      <c r="A11" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
       <c r="A12" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A13" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A14" s="1"/>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A15" s="25" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A16" s="25" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A17" s="25" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A19" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="B26" s="1"/>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="B27" s="2"/>
+    <row r="13" spans="1:2">
+      <c r="A13" s="1"/>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" s="21" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15" s="21" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
+      <c r="A16" s="21" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2">
+      <c r="B25" s="1"/>
+    </row>
+    <row r="26" spans="1:2">
+      <c r="B26" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="B8" r:id="rId1" xr:uid="{A48EA53C-1AB9-44F3-861F-8B55FB21C4C2}"/>
+    <hyperlink ref="B8" r:id="rId1" xr:uid="{4078C656-C4AE-4A6F-8793-A09E7B4DF1DF}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId2"/>
@@ -788,12 +843,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:AZ20"/>
-  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:52" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:52">
       <c r="A1" s="1"/>
       <c r="D1" s="1"/>
       <c r="G1" s="1"/>
@@ -813,46 +868,48 @@
       <c r="AW1" s="1"/>
       <c r="AZ1" s="1"/>
     </row>
-    <row r="2" spans="1:52" ht="27.6" x14ac:dyDescent="0.6">
+    <row r="2" spans="1:52" ht="23.5">
       <c r="B2" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:52" ht="25.5" customHeight="1">
+      <c r="B3" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" s="15"/>
+      <c r="D3" s="15"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="16"/>
+      <c r="G3" s="16"/>
+      <c r="H3" t="s">
+        <v>26</v>
+      </c>
+      <c r="T3" s="24"/>
+      <c r="W3" s="12" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:52" s="7" customFormat="1">
+      <c r="A4" s="7" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="3" spans="1:52" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B3" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" s="17"/>
-      <c r="D3" s="17"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
-      <c r="T3" s="23"/>
-      <c r="U3" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="V3" s="13"/>
-      <c r="W3" s="13"/>
-    </row>
-    <row r="4" spans="1:52" s="7" customFormat="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" s="16">
+      <c r="B4" s="14">
         <v>2018</v>
       </c>
-      <c r="C4" s="16">
+      <c r="C4" s="14">
         <v>2019</v>
       </c>
-      <c r="D4" s="7">
+      <c r="D4" s="14">
         <v>2020</v>
       </c>
-      <c r="E4" s="7">
+      <c r="E4" s="14">
         <v>2021</v>
       </c>
-      <c r="F4" s="7">
+      <c r="F4" s="14">
         <v>2022</v>
       </c>
-      <c r="G4" s="7">
+      <c r="G4" s="14">
         <v>2023</v>
       </c>
       <c r="H4" s="7">
@@ -888,312 +945,318 @@
       <c r="R4" s="7">
         <v>2034</v>
       </c>
-      <c r="S4" s="14">
+      <c r="S4" s="7">
         <v>2035</v>
       </c>
-      <c r="T4" s="14">
+      <c r="T4" s="7">
         <v>2036</v>
       </c>
-      <c r="U4" s="14">
+      <c r="U4" s="7">
         <v>2037</v>
       </c>
-      <c r="V4" s="14">
+      <c r="V4" s="7">
         <v>2038</v>
       </c>
-      <c r="W4" s="14">
+      <c r="W4" s="13">
         <v>2039</v>
       </c>
-      <c r="X4" s="14">
+      <c r="X4" s="13">
         <v>2040</v>
       </c>
-      <c r="Y4" s="14">
+      <c r="Y4" s="13">
         <v>2041</v>
       </c>
-      <c r="Z4" s="14">
+      <c r="Z4" s="13">
         <v>2042</v>
       </c>
-      <c r="AA4" s="14">
+      <c r="AA4" s="13">
         <v>2043</v>
       </c>
-      <c r="AB4" s="14">
+      <c r="AB4" s="13">
         <v>2044</v>
       </c>
-      <c r="AC4" s="14">
+      <c r="AC4" s="13">
         <v>2045</v>
       </c>
-      <c r="AD4" s="14">
+      <c r="AD4" s="13">
         <v>2046</v>
       </c>
-      <c r="AE4" s="14">
+      <c r="AE4" s="13">
         <v>2047</v>
       </c>
-      <c r="AF4" s="14">
+      <c r="AF4" s="13">
         <v>2048</v>
       </c>
-      <c r="AG4" s="14">
+      <c r="AG4" s="13">
         <v>2049</v>
       </c>
-      <c r="AH4" s="14">
+      <c r="AH4" s="13">
         <v>2050</v>
       </c>
     </row>
-    <row r="5" spans="1:52" s="7" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:52" s="7" customFormat="1" ht="17">
       <c r="A5" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="14">
+        <f>C5/(1+$I$6)</f>
+        <v>2230.3920030879835</v>
+      </c>
+      <c r="C5" s="14">
+        <f>D5/(1+$I$6)</f>
+        <v>2319.0378172632331</v>
+      </c>
+      <c r="D5" s="14">
+        <f t="shared" ref="D5:G5" si="0">E5/(1+$I$6)</f>
+        <v>2411.2068149685142</v>
+      </c>
+      <c r="E5" s="14">
+        <f t="shared" si="0"/>
+        <v>2507.0390233703856</v>
+      </c>
+      <c r="F5" s="14">
+        <f t="shared" si="0"/>
+        <v>2606.6800349450778</v>
+      </c>
+      <c r="G5" s="14">
+        <f t="shared" si="0"/>
+        <v>2710.2812286689418</v>
+      </c>
+      <c r="H5" s="25">
+        <v>2818</v>
+      </c>
+      <c r="I5" s="26">
+        <v>2930</v>
+      </c>
+      <c r="J5" s="26">
+        <v>3053</v>
+      </c>
+      <c r="K5" s="25">
+        <v>3190</v>
+      </c>
+      <c r="L5" s="26">
+        <v>3319</v>
+      </c>
+      <c r="M5" s="26">
+        <v>3416</v>
+      </c>
+      <c r="N5" s="25">
+        <v>3532</v>
+      </c>
+      <c r="O5" s="26">
+        <v>3653</v>
+      </c>
+      <c r="P5" s="26">
+        <v>3788</v>
+      </c>
+      <c r="Q5" s="25">
+        <v>3926</v>
+      </c>
+      <c r="R5" s="26">
+        <v>4071</v>
+      </c>
+      <c r="S5" s="26">
+        <v>4234</v>
+      </c>
+      <c r="T5" s="25">
+        <v>4374</v>
+      </c>
+      <c r="U5" s="26">
+        <v>4529</v>
+      </c>
+      <c r="V5" s="25">
+        <v>4692</v>
+      </c>
+      <c r="W5" s="7">
+        <f>V5*(1+$V$6)</f>
+        <v>4860.8664164274669</v>
+      </c>
+      <c r="X5" s="7">
+        <f t="shared" ref="X5:AH5" si="1">W5*(1+$V$6)</f>
+        <v>5035.8103832805637</v>
+      </c>
+      <c r="Y5" s="7">
+        <f t="shared" si="1"/>
+        <v>5217.0506333301837</v>
+      </c>
+      <c r="Z5" s="7">
+        <f t="shared" si="1"/>
+        <v>5404.8137716019473</v>
+      </c>
+      <c r="AA5" s="7">
+        <f t="shared" si="1"/>
+        <v>5599.3345587008907</v>
+      </c>
+      <c r="AB5" s="7">
+        <f t="shared" si="1"/>
+        <v>5800.856204333093</v>
+      </c>
+      <c r="AC5" s="7">
+        <f t="shared" si="1"/>
+        <v>6009.6306713912281</v>
+      </c>
+      <c r="AD5" s="7">
+        <f t="shared" si="1"/>
+        <v>6225.9189909842435</v>
+      </c>
+      <c r="AE5" s="7">
+        <f t="shared" si="1"/>
+        <v>6449.9915888050491</v>
+      </c>
+      <c r="AF5" s="7">
+        <f t="shared" si="1"/>
+        <v>6682.1286232442681</v>
+      </c>
+      <c r="AG5" s="7">
+        <f t="shared" si="1"/>
+        <v>6922.6203356727983</v>
+      </c>
+      <c r="AH5" s="7">
+        <f t="shared" si="1"/>
+        <v>7171.7674133311475</v>
+      </c>
+    </row>
+    <row r="6" spans="1:52" s="7" customFormat="1">
+      <c r="A6" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="16">
-        <f>C5/(1+$E$6)</f>
-        <v>2194.7069996712471</v>
-      </c>
-      <c r="C5" s="16">
-        <f>D5/(1+$E$6)</f>
-        <v>2312.6826323987539</v>
-      </c>
-      <c r="D5" s="22">
-        <v>2437</v>
-      </c>
-      <c r="E5" s="22">
-        <v>2568</v>
-      </c>
-      <c r="F5" s="22">
-        <v>2947</v>
-      </c>
-      <c r="G5" s="22">
-        <v>3018</v>
-      </c>
-      <c r="H5" s="22">
-        <v>3141</v>
-      </c>
-      <c r="I5" s="22">
-        <v>3258</v>
-      </c>
-      <c r="J5" s="22">
-        <v>3361</v>
-      </c>
-      <c r="K5" s="22">
-        <v>3483</v>
-      </c>
-      <c r="L5" s="22">
-        <v>3673</v>
-      </c>
-      <c r="M5" s="22">
-        <v>3865</v>
-      </c>
-      <c r="N5" s="22">
-        <v>4057</v>
-      </c>
-      <c r="O5" s="22">
-        <v>4271</v>
-      </c>
-      <c r="P5" s="22">
-        <v>4488</v>
-      </c>
-      <c r="Q5" s="22">
-        <v>4711</v>
-      </c>
-      <c r="R5" s="22">
-        <v>4935</v>
-      </c>
-      <c r="S5" s="22">
-        <v>5025</v>
-      </c>
-      <c r="T5" s="22">
-        <v>5136</v>
-      </c>
-      <c r="U5" s="7">
-        <f>T5*(1+$T$6)</f>
-        <v>5249.4519402985079</v>
-      </c>
-      <c r="V5" s="7">
-        <f>U5*(1+$T$6)</f>
-        <v>5365.4099831588337</v>
-      </c>
-      <c r="W5" s="7">
-        <f>V5*(1+$T$6)</f>
-        <v>5483.9294872644323</v>
-      </c>
-      <c r="X5" s="7">
-        <f t="shared" ref="X5:AH5" si="0">W5*(1+$T$6)</f>
-        <v>5605.0670341472887</v>
-      </c>
-      <c r="Y5" s="7">
-        <f t="shared" si="0"/>
-        <v>5728.8804552000947</v>
-      </c>
-      <c r="Z5" s="7">
-        <f t="shared" si="0"/>
-        <v>5855.4288592851126</v>
-      </c>
-      <c r="AA5" s="7">
-        <f t="shared" si="0"/>
-        <v>5984.7726609529036</v>
-      </c>
-      <c r="AB5" s="7">
-        <f t="shared" si="0"/>
-        <v>6116.9736092844014</v>
-      </c>
-      <c r="AC5" s="7">
-        <f t="shared" si="0"/>
-        <v>6252.0948173700872</v>
-      </c>
-      <c r="AD5" s="7">
-        <f t="shared" si="0"/>
-        <v>6390.2007924403524</v>
-      </c>
-      <c r="AE5" s="7">
-        <f t="shared" si="0"/>
-        <v>6531.3574666614231</v>
-      </c>
-      <c r="AF5" s="7">
-        <f t="shared" si="0"/>
-        <v>6675.6322286115565</v>
-      </c>
-      <c r="AG5" s="7">
-        <f t="shared" si="0"/>
-        <v>6823.0939554525285</v>
-      </c>
-      <c r="AH5" s="7">
-        <f t="shared" si="0"/>
-        <v>6973.8130458117785</v>
-      </c>
-    </row>
-    <row r="6" spans="1:52" s="7" customFormat="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="7" t="s">
+      <c r="B6" s="14"/>
+      <c r="C6" s="14"/>
+      <c r="D6" s="8" t="s">
         <v>14</v>
-      </c>
-      <c r="B6" s="16"/>
-      <c r="C6" s="16"/>
-      <c r="D6" s="8" t="s">
-        <v>15</v>
       </c>
       <c r="E6" s="7">
         <f>(E5-D5)/D5</f>
-        <v>5.3754616331555191E-2</v>
+        <v>3.9744499645138404E-2</v>
       </c>
       <c r="F6" s="7">
-        <f t="shared" ref="F6:R6" si="1">(F5-E5)/E5</f>
-        <v>0.14758566978193147</v>
+        <f t="shared" ref="F6:R6" si="2">(F5-E5)/E5</f>
+        <v>3.9744499645138286E-2</v>
       </c>
       <c r="G6" s="7">
-        <f t="shared" si="1"/>
-        <v>2.4092297251442144E-2</v>
+        <f t="shared" si="2"/>
+        <v>3.9744499645138431E-2</v>
       </c>
       <c r="H6" s="7">
-        <f t="shared" si="1"/>
-        <v>4.0755467196819085E-2</v>
+        <f t="shared" si="2"/>
+        <v>3.9744499645138459E-2</v>
       </c>
       <c r="I6" s="7">
-        <f t="shared" si="1"/>
-        <v>3.7249283667621778E-2</v>
+        <f t="shared" si="2"/>
+        <v>3.9744499645138397E-2</v>
       </c>
       <c r="J6" s="7">
-        <f t="shared" si="1"/>
-        <v>3.1614487415592391E-2</v>
+        <f t="shared" si="2"/>
+        <v>4.1979522184300344E-2</v>
       </c>
       <c r="K6" s="7">
-        <f t="shared" si="1"/>
-        <v>3.6298720618863432E-2</v>
+        <f t="shared" si="2"/>
+        <v>4.4873894529970523E-2</v>
       </c>
       <c r="L6" s="7">
-        <f t="shared" si="1"/>
-        <v>5.4550674705713467E-2</v>
+        <f t="shared" si="2"/>
+        <v>4.0438871473354232E-2</v>
       </c>
       <c r="M6" s="7">
-        <f t="shared" si="1"/>
-        <v>5.2273346038660497E-2</v>
+        <f t="shared" si="2"/>
+        <v>2.9225670382645376E-2</v>
       </c>
       <c r="N6" s="7">
-        <f t="shared" si="1"/>
-        <v>4.9676584734799481E-2</v>
+        <f t="shared" si="2"/>
+        <v>3.3957845433255272E-2</v>
       </c>
       <c r="O6" s="7">
-        <f t="shared" si="1"/>
-        <v>5.2748336209021446E-2</v>
+        <f t="shared" si="2"/>
+        <v>3.4258210645526616E-2</v>
       </c>
       <c r="P6" s="7">
-        <f t="shared" si="1"/>
-        <v>5.0807773355186138E-2</v>
+        <f t="shared" si="2"/>
+        <v>3.6955926635641935E-2</v>
       </c>
       <c r="Q6" s="7">
-        <f t="shared" si="1"/>
-        <v>4.9688057040998219E-2</v>
+        <f t="shared" si="2"/>
+        <v>3.6430834213305174E-2</v>
       </c>
       <c r="R6" s="7">
-        <f t="shared" si="1"/>
-        <v>4.7548291233283801E-2</v>
-      </c>
-      <c r="S6" s="14">
-        <f t="shared" ref="S6" si="2">(S5-R5)/R5</f>
-        <v>1.82370820668693E-2</v>
-      </c>
-      <c r="T6" s="14">
-        <f t="shared" ref="T6" si="3">(T5-S5)/S5</f>
-        <v>2.208955223880597E-2</v>
-      </c>
-      <c r="U6" s="14">
-        <f t="shared" ref="U6" si="4">(U5-T5)/T5</f>
-        <v>2.2089552238806057E-2</v>
-      </c>
-      <c r="V6" s="14">
-        <f t="shared" ref="V6" si="5">(V5-U5)/U5</f>
-        <v>2.2089552238806077E-2</v>
-      </c>
-      <c r="W6" s="14">
-        <f t="shared" ref="W6" si="6">(W5-V5)/V5</f>
-        <v>2.2089552238806053E-2</v>
-      </c>
-      <c r="X6" s="14">
-        <f t="shared" ref="X6" si="7">(X5-W5)/W5</f>
-        <v>2.2089552238806029E-2</v>
-      </c>
-      <c r="Y6" s="14">
-        <f t="shared" ref="Y6" si="8">(Y5-X5)/X5</f>
-        <v>2.2089552238806012E-2</v>
-      </c>
-      <c r="Z6" s="14">
-        <f t="shared" ref="Z6" si="9">(Z5-Y5)/Y5</f>
-        <v>2.2089552238806119E-2</v>
-      </c>
-      <c r="AA6" s="14">
-        <f t="shared" ref="AA6" si="10">(AA5-Z5)/Z5</f>
-        <v>2.208955223880605E-2</v>
-      </c>
-      <c r="AB6" s="14">
-        <f t="shared" ref="AB6" si="11">(AB5-AA5)/AA5</f>
-        <v>2.2089552238806105E-2</v>
-      </c>
-      <c r="AC6" s="14">
-        <f t="shared" ref="AC6" si="12">(AC5-AB5)/AB5</f>
-        <v>2.2089552238806053E-2</v>
-      </c>
-      <c r="AD6" s="14">
-        <f t="shared" ref="AD6" si="13">(AD5-AC5)/AC5</f>
-        <v>2.2089552238806071E-2</v>
-      </c>
-      <c r="AE6" s="14">
-        <f t="shared" ref="AE6" si="14">(AE5-AD5)/AD5</f>
-        <v>2.2089552238806008E-2</v>
-      </c>
-      <c r="AF6" s="14">
-        <f t="shared" ref="AF6" si="15">(AF5-AE5)/AE5</f>
-        <v>2.2089552238806032E-2</v>
-      </c>
-      <c r="AG6" s="14">
-        <f t="shared" ref="AG6" si="16">(AG5-AF5)/AF5</f>
-        <v>2.2089552238806015E-2</v>
-      </c>
-      <c r="AH6" s="14">
-        <f t="shared" ref="AH6" si="17">(AH5-AG5)/AG5</f>
-        <v>2.2089552238805987E-2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:52" s="7" customFormat="1" x14ac:dyDescent="0.4"/>
-    <row r="8" spans="1:52" s="7" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v>3.6933265410086603E-2</v>
+      </c>
+      <c r="S6" s="7">
+        <f t="shared" ref="S6" si="3">(S5-R5)/R5</f>
+        <v>4.0039302382706948E-2</v>
+      </c>
+      <c r="T6" s="7">
+        <f t="shared" ref="T6" si="4">(T5-S5)/S5</f>
+        <v>3.3065658951346243E-2</v>
+      </c>
+      <c r="U6" s="7">
+        <f t="shared" ref="U6" si="5">(U5-T5)/T5</f>
+        <v>3.5436671239140377E-2</v>
+      </c>
+      <c r="V6" s="7">
+        <f t="shared" ref="V6" si="6">(V5-U5)/U5</f>
+        <v>3.5990284831088543E-2</v>
+      </c>
+      <c r="W6" s="13">
+        <f t="shared" ref="W6" si="7">(W5-V5)/V5</f>
+        <v>3.5990284831088425E-2</v>
+      </c>
+      <c r="X6" s="13">
+        <f t="shared" ref="X6" si="8">(X5-W5)/W5</f>
+        <v>3.5990284831088452E-2</v>
+      </c>
+      <c r="Y6" s="13">
+        <f t="shared" ref="Y6" si="9">(Y5-X5)/X5</f>
+        <v>3.5990284831088425E-2</v>
+      </c>
+      <c r="Z6" s="13">
+        <f t="shared" ref="Z6" si="10">(Z5-Y5)/Y5</f>
+        <v>3.5990284831088439E-2</v>
+      </c>
+      <c r="AA6" s="13">
+        <f t="shared" ref="AA6" si="11">(AA5-Z5)/Z5</f>
+        <v>3.5990284831088432E-2</v>
+      </c>
+      <c r="AB6" s="13">
+        <f t="shared" ref="AB6" si="12">(AB5-AA5)/AA5</f>
+        <v>3.5990284831088501E-2</v>
+      </c>
+      <c r="AC6" s="13">
+        <f t="shared" ref="AC6" si="13">(AC5-AB5)/AB5</f>
+        <v>3.5990284831088529E-2</v>
+      </c>
+      <c r="AD6" s="13">
+        <f t="shared" ref="AD6" si="14">(AD5-AC5)/AC5</f>
+        <v>3.5990284831088404E-2</v>
+      </c>
+      <c r="AE6" s="13">
+        <f t="shared" ref="AE6" si="15">(AE5-AD5)/AD5</f>
+        <v>3.5990284831088439E-2</v>
+      </c>
+      <c r="AF6" s="13">
+        <f t="shared" ref="AF6" si="16">(AF5-AE5)/AE5</f>
+        <v>3.5990284831088529E-2</v>
+      </c>
+      <c r="AG6" s="13">
+        <f t="shared" ref="AG6" si="17">(AG5-AF5)/AF5</f>
+        <v>3.5990284831088473E-2</v>
+      </c>
+      <c r="AH6" s="13">
+        <f t="shared" ref="AH6" si="18">(AH5-AG5)/AG5</f>
+        <v>3.5990284831088459E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:52" s="7" customFormat="1">
+      <c r="W7" s="19" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:52" s="7" customFormat="1" ht="16.5" customHeight="1">
       <c r="A8" s="9"/>
-      <c r="B8" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="C8" s="20"/>
+      <c r="B8" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" s="18"/>
       <c r="D8" s="11"/>
       <c r="E8" s="11"/>
       <c r="F8" s="11"/>
@@ -1209,53 +1272,49 @@
       <c r="P8" s="11"/>
       <c r="Q8" s="10"/>
       <c r="R8" s="11"/>
-      <c r="S8" s="21" t="s">
-        <v>17</v>
-      </c>
-      <c r="T8" s="14"/>
-    </row>
-    <row r="9" spans="1:52" s="7" customFormat="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="9" spans="1:52" s="7" customFormat="1">
       <c r="A9" s="5" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="10" spans="1:52" s="7" customFormat="1" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:52" s="7" customFormat="1">
       <c r="A10"/>
     </row>
-    <row r="11" spans="1:52" s="7" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:52" s="7" customFormat="1">
       <c r="A11"/>
     </row>
-    <row r="12" spans="1:52" s="7" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:52" s="7" customFormat="1">
       <c r="A12"/>
     </row>
-    <row r="13" spans="1:52" s="7" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:52" s="7" customFormat="1">
       <c r="A13"/>
     </row>
-    <row r="14" spans="1:52" s="7" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:52" s="7" customFormat="1">
       <c r="A14" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="15" spans="1:52" s="7" customFormat="1" x14ac:dyDescent="0.4">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="15" spans="1:52" s="7" customFormat="1">
       <c r="A15"/>
     </row>
-    <row r="16" spans="1:52" s="7" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:52" s="7" customFormat="1">
       <c r="A16" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" s="7" customFormat="1" x14ac:dyDescent="0.4">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" s="7" customFormat="1">
       <c r="A17"/>
     </row>
-    <row r="18" spans="1:1" s="7" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:1" s="7" customFormat="1">
       <c r="A18"/>
     </row>
-    <row r="19" spans="1:1" s="7" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:1" s="7" customFormat="1">
       <c r="A19" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" s="7" customFormat="1" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" s="7" customFormat="1">
       <c r="A20">
         <v>4</v>
       </c>
@@ -1264,6 +1323,7 @@
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -1273,12 +1333,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AH2"/>
-  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="19.19921875" customWidth="1"/>
+    <col min="1" max="1" width="19.08984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:34">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1382,141 +1442,141 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:34" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:34">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="7">
         <f>MOTIE!B5</f>
-        <v>2194.7069996712471</v>
+        <v>2230.3920030879835</v>
       </c>
       <c r="C2" s="7">
         <f>MOTIE!C5</f>
-        <v>2312.6826323987539</v>
+        <v>2319.0378172632331</v>
       </c>
       <c r="D2" s="7">
         <f>MOTIE!D5</f>
-        <v>2437</v>
+        <v>2411.2068149685142</v>
       </c>
       <c r="E2" s="3">
         <f>MOTIE!E5</f>
-        <v>2568</v>
+        <v>2507.0390233703856</v>
       </c>
       <c r="F2" s="3">
         <f>MOTIE!F5</f>
-        <v>2947</v>
+        <v>2606.6800349450778</v>
       </c>
       <c r="G2" s="3">
         <f>MOTIE!G5</f>
-        <v>3018</v>
+        <v>2710.2812286689418</v>
       </c>
       <c r="H2" s="3">
         <f>MOTIE!H5</f>
-        <v>3141</v>
+        <v>2818</v>
       </c>
       <c r="I2" s="3">
         <f>MOTIE!I5</f>
-        <v>3258</v>
+        <v>2930</v>
       </c>
       <c r="J2" s="3">
         <f>MOTIE!J5</f>
-        <v>3361</v>
+        <v>3053</v>
       </c>
       <c r="K2" s="3">
         <f>MOTIE!K5</f>
-        <v>3483</v>
+        <v>3190</v>
       </c>
       <c r="L2" s="3">
         <f>MOTIE!L5</f>
-        <v>3673</v>
+        <v>3319</v>
       </c>
       <c r="M2" s="3">
         <f>MOTIE!M5</f>
-        <v>3865</v>
+        <v>3416</v>
       </c>
       <c r="N2" s="3">
         <f>MOTIE!N5</f>
-        <v>4057</v>
+        <v>3532</v>
       </c>
       <c r="O2" s="3">
         <f>MOTIE!O5</f>
-        <v>4271</v>
+        <v>3653</v>
       </c>
       <c r="P2" s="3">
         <f>MOTIE!P5</f>
-        <v>4488</v>
+        <v>3788</v>
       </c>
       <c r="Q2" s="3">
         <f>MOTIE!Q5</f>
-        <v>4711</v>
+        <v>3926</v>
       </c>
       <c r="R2" s="3">
         <f>MOTIE!R5</f>
-        <v>4935</v>
+        <v>4071</v>
       </c>
       <c r="S2" s="3">
         <f>MOTIE!S5</f>
-        <v>5025</v>
+        <v>4234</v>
       </c>
       <c r="T2" s="3">
         <f>MOTIE!T5</f>
-        <v>5136</v>
+        <v>4374</v>
       </c>
       <c r="U2" s="3">
         <f>MOTIE!U5</f>
-        <v>5249.4519402985079</v>
+        <v>4529</v>
       </c>
       <c r="V2" s="3">
         <f>MOTIE!V5</f>
-        <v>5365.4099831588337</v>
+        <v>4692</v>
       </c>
       <c r="W2" s="3">
         <f>MOTIE!W5</f>
-        <v>5483.9294872644323</v>
+        <v>4860.8664164274669</v>
       </c>
       <c r="X2" s="3">
         <f>MOTIE!X5</f>
-        <v>5605.0670341472887</v>
+        <v>5035.8103832805637</v>
       </c>
       <c r="Y2" s="3">
         <f>MOTIE!Y5</f>
-        <v>5728.8804552000947</v>
+        <v>5217.0506333301837</v>
       </c>
       <c r="Z2" s="3">
         <f>MOTIE!Z5</f>
-        <v>5855.4288592851126</v>
+        <v>5404.8137716019473</v>
       </c>
       <c r="AA2" s="3">
         <f>MOTIE!AA5</f>
-        <v>5984.7726609529036</v>
+        <v>5599.3345587008907</v>
       </c>
       <c r="AB2" s="3">
         <f>MOTIE!AB5</f>
-        <v>6116.9736092844014</v>
+        <v>5800.856204333093</v>
       </c>
       <c r="AC2" s="3">
         <f>MOTIE!AC5</f>
-        <v>6252.0948173700872</v>
+        <v>6009.6306713912281</v>
       </c>
       <c r="AD2" s="3">
         <f>MOTIE!AD5</f>
-        <v>6390.2007924403524</v>
+        <v>6225.9189909842435</v>
       </c>
       <c r="AE2" s="3">
         <f>MOTIE!AE5</f>
-        <v>6531.3574666614231</v>
+        <v>6449.9915888050491</v>
       </c>
       <c r="AF2" s="3">
         <f>MOTIE!AF5</f>
-        <v>6675.6322286115565</v>
+        <v>6682.1286232442681</v>
       </c>
       <c r="AG2" s="3">
         <f>MOTIE!AG5</f>
-        <v>6823.0939554525285</v>
+        <v>6922.6203356727983</v>
       </c>
       <c r="AH2" s="3">
         <f>MOTIE!AH5</f>
-        <v>6973.8130458117785</v>
+        <v>7171.7674133311475</v>
       </c>
     </row>
   </sheetData>
@@ -1531,12 +1591,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AH2"/>
-  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:34">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1640,140 +1700,141 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:34" ht="34.799999999999997" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:34" ht="29">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3">
-        <f>C2</f>
-        <v>0</v>
-      </c>
-      <c r="C2" s="3">
+      <c r="B2" s="3" cm="1">
+        <f t="array" ref="B2">_xlfn.SINGLE(IF((TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!B1)-'DRC-BDRC'!B2)&gt;0,(TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!B1)-'DRC-BDRC'!B2),0))</f>
+        <v>0</v>
+      </c>
+      <c r="C2" s="3" cm="1">
+        <f t="array" ref="C2">_xlfn.SINGLE(IF((TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!C1)-'DRC-BDRC'!C2)&gt;0,(TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!C1)-'DRC-BDRC'!C2),0))</f>
         <v>0</v>
       </c>
       <c r="D2" s="3" cm="1">
-        <f t="array" ref="D2">_xlfn.SINGLE(IF((TREND(MOTIE!$E$5:$Q$5,MOTIE!$E$4:$Q$4,'DRC-PADRC'!D1)-'DRC-BDRC'!D2)&gt;0,(TREND(MOTIE!$E$5:$Q$5,MOTIE!$E$4:$Q$4,'DRC-PADRC'!D1)-'DRC-BDRC'!D2),0))</f>
-        <v>18.11538461537566</v>
+        <f t="array" ref="D2">_xlfn.SINGLE(IF((TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!D1)-'DRC-BDRC'!D2)&gt;0,(TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!D1)-'DRC-BDRC'!D2),0))</f>
+        <v>0</v>
       </c>
       <c r="E2" s="3" cm="1">
-        <f t="array" ref="E2">_xlfn.SINGLE(IF((TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!E1)-'DRC-BDRC'!E2)&gt;0,(TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!E1)-'DRC-BDRC'!E2),0))</f>
-        <v>25.580882352951448</v>
+        <f t="array" ref="E2">_xlfn.SINGLE(IF((TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!E1)-'DRC-BDRC'!E2)&gt;0,(TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!E1)-'DRC-BDRC'!E2),0))</f>
+        <v>0</v>
       </c>
       <c r="F2" s="3" cm="1">
-        <f t="array" ref="F2">_xlfn.SINGLE(IF((TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!F1)-'DRC-BDRC'!F2)&gt;0,(TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!F1)-'DRC-BDRC'!F2),0))</f>
+        <f t="array" ref="F2">_xlfn.SINGLE(IF((TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!F1)-'DRC-BDRC'!F2)&gt;0,(TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!F1)-'DRC-BDRC'!F2),0))</f>
         <v>0</v>
       </c>
       <c r="G2" s="3" cm="1">
-        <f t="array" ref="G2">_xlfn.SINGLE(IF((TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!G1)-'DRC-BDRC'!G2)&gt;0,(TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!G1)-'DRC-BDRC'!G2),0))</f>
+        <f t="array" ref="G2">_xlfn.SINGLE(IF((TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!G1)-'DRC-BDRC'!G2)&gt;0,(TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!G1)-'DRC-BDRC'!G2),0))</f>
         <v>0</v>
       </c>
       <c r="H2" s="3" cm="1">
-        <f t="array" ref="H2">_xlfn.SINGLE(IF((TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!H1)-'DRC-BDRC'!H2)&gt;0,(TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!H1)-'DRC-BDRC'!H2),0))</f>
+        <f t="array" ref="H2">_xlfn.SINGLE(IF((TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!H1)-'DRC-BDRC'!H2)&gt;0,(TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!H1)-'DRC-BDRC'!H2),0))</f>
         <v>0</v>
       </c>
       <c r="I2" s="3" cm="1">
-        <f t="array" ref="I2">_xlfn.SINGLE(IF((TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!I1)-'DRC-BDRC'!I2)&gt;0,(TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!I1)-'DRC-BDRC'!I2),0))</f>
-        <v>16.904411764699034</v>
+        <f t="array" ref="I2">_xlfn.SINGLE(IF((TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!I1)-'DRC-BDRC'!I2)&gt;0,(TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!I1)-'DRC-BDRC'!I2),0))</f>
+        <v>0</v>
       </c>
       <c r="J2" s="3" cm="1">
-        <f t="array" ref="J2">_xlfn.SINGLE(IF((TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!J1)-'DRC-BDRC'!J2)&gt;0,(TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!J1)-'DRC-BDRC'!J2),0))</f>
-        <v>84.235294117650483</v>
+        <f t="array" ref="J2">_xlfn.SINGLE(IF((TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!J1)-'DRC-BDRC'!J2)&gt;0,(TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!J1)-'DRC-BDRC'!J2),0))</f>
+        <v>0</v>
       </c>
       <c r="K2" s="3" cm="1">
-        <f t="array" ref="K2">_xlfn.SINGLE(IF((TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!K1)-'DRC-BDRC'!K2)&gt;0,(TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!K1)-'DRC-BDRC'!K2),0))</f>
-        <v>132.56617647060193</v>
+        <f t="array" ref="K2">_xlfn.SINGLE(IF((TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!K1)-'DRC-BDRC'!K2)&gt;0,(TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!K1)-'DRC-BDRC'!K2),0))</f>
+        <v>0</v>
       </c>
       <c r="L2" s="3" cm="1">
-        <f t="array" ref="L2">_xlfn.SINGLE(IF((TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!L1)-'DRC-BDRC'!L2)&gt;0,(TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!L1)-'DRC-BDRC'!L2),0))</f>
-        <v>112.89705882355338</v>
+        <f t="array" ref="L2">_xlfn.SINGLE(IF((TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!L1)-'DRC-BDRC'!L2)&gt;0,(TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!L1)-'DRC-BDRC'!L2),0))</f>
+        <v>0</v>
       </c>
       <c r="M2" s="3" cm="1">
-        <f t="array" ref="M2">_xlfn.SINGLE(IF((TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!M1)-'DRC-BDRC'!M2)&gt;0,(TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!M1)-'DRC-BDRC'!M2),0))</f>
-        <v>91.22794117644662</v>
+        <f t="array" ref="M2">_xlfn.SINGLE(IF((TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!M1)-'DRC-BDRC'!M2)&gt;0,(TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!M1)-'DRC-BDRC'!M2),0))</f>
+        <v>21.202380952367093</v>
       </c>
       <c r="N2" s="3" cm="1">
-        <f t="array" ref="N2">_xlfn.SINGLE(IF((TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!N1)-'DRC-BDRC'!N2)&gt;0,(TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!N1)-'DRC-BDRC'!N2),0))</f>
-        <v>69.558823529398069</v>
+        <f t="array" ref="N2">_xlfn.SINGLE(IF((TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!N1)-'DRC-BDRC'!N2)&gt;0,(TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!N1)-'DRC-BDRC'!N2),0))</f>
+        <v>37.434523809526581</v>
       </c>
       <c r="O2" s="3" cm="1">
-        <f t="array" ref="O2">_xlfn.SINGLE(IF((TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!O1)-'DRC-BDRC'!O2)&gt;0,(TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!O1)-'DRC-BDRC'!O2),0))</f>
-        <v>25.889705882349517</v>
+        <f t="array" ref="O2">_xlfn.SINGLE(IF((TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!O1)-'DRC-BDRC'!O2)&gt;0,(TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!O1)-'DRC-BDRC'!O2),0))</f>
+        <v>48.666666666686069</v>
       </c>
       <c r="P2" s="3" cm="1">
-        <f t="array" ref="P2">_xlfn.SINGLE(IF((TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!P1)-'DRC-BDRC'!P2)&gt;0,(TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!P1)-'DRC-BDRC'!P2),0))</f>
-        <v>0</v>
+        <f t="array" ref="P2">_xlfn.SINGLE(IF((TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!P1)-'DRC-BDRC'!P2)&gt;0,(TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!P1)-'DRC-BDRC'!P2),0))</f>
+        <v>45.898809523845557</v>
       </c>
       <c r="Q2" s="3" cm="1">
-        <f t="array" ref="Q2">_xlfn.SINGLE(IF((TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!Q1)-'DRC-BDRC'!Q2)&gt;0,(TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!Q1)-'DRC-BDRC'!Q2),0))</f>
-        <v>0</v>
+        <f t="array" ref="Q2">_xlfn.SINGLE(IF((TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!Q1)-'DRC-BDRC'!Q2)&gt;0,(TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!Q1)-'DRC-BDRC'!Q2),0))</f>
+        <v>40.130952380946837</v>
       </c>
       <c r="R2" s="3" cm="1">
-        <f t="array" ref="R2">_xlfn.SINGLE(IF((TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!R1)-'DRC-BDRC'!R2)&gt;0,(TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!R1)-'DRC-BDRC'!R2),0))</f>
-        <v>0</v>
+        <f t="array" ref="R2">_xlfn.SINGLE(IF((TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!R1)-'DRC-BDRC'!R2)&gt;0,(TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!R1)-'DRC-BDRC'!R2),0))</f>
+        <v>27.363095238106325</v>
       </c>
       <c r="S2" s="3" cm="1">
-        <f t="array" ref="S2">_xlfn.SINGLE(IF((TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!S1)-'DRC-BDRC'!S2)&gt;0,(TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!S1)-'DRC-BDRC'!S2),0))</f>
+        <f t="array" ref="S2">_xlfn.SINGLE(IF((TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!S1)-'DRC-BDRC'!S2)&gt;0,(TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!S1)-'DRC-BDRC'!S2),0))</f>
         <v>0</v>
       </c>
       <c r="T2" s="3" cm="1">
-        <f t="array" ref="T2">_xlfn.SINGLE(IF((TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!T1)-'DRC-BDRC'!T2)&gt;0,(TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!T1)-'DRC-BDRC'!T2),0))</f>
-        <v>12.544117647048552</v>
+        <f t="array" ref="T2">_xlfn.SINGLE(IF((TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!T1)-'DRC-BDRC'!T2)&gt;0,(TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!T1)-'DRC-BDRC'!T2),0))</f>
+        <v>0</v>
       </c>
       <c r="U2" s="3" cm="1">
-        <f t="array" ref="U2">_xlfn.SINGLE(IF((TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!U1)-'DRC-BDRC'!U2)&gt;0,(TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!U1)-'DRC-BDRC'!U2),0))</f>
-        <v>69.423059701492093</v>
+        <f t="array" ref="U2">_xlfn.SINGLE(IF((TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!U1)-'DRC-BDRC'!U2)&gt;0,(TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!U1)-'DRC-BDRC'!U2),0))</f>
+        <v>0</v>
       </c>
       <c r="V2" s="3" cm="1">
-        <f t="array" ref="V2">_xlfn.SINGLE(IF((TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!V1)-'DRC-BDRC'!V2)&gt;0,(TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!V1)-'DRC-BDRC'!V2),0))</f>
-        <v>123.79589919411774</v>
+        <f t="array" ref="V2">_xlfn.SINGLE(IF((TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!V1)-'DRC-BDRC'!V2)&gt;0,(TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!V1)-'DRC-BDRC'!V2),0))</f>
+        <v>0</v>
       </c>
       <c r="W2" s="3" cm="1">
-        <f t="array" ref="W2">_xlfn.SINGLE(IF((TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!W1)-'DRC-BDRC'!W2)&gt;0,(TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!W1)-'DRC-BDRC'!W2),0))</f>
-        <v>175.60727744147061</v>
+        <f t="array" ref="W2">_xlfn.SINGLE(IF((TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!W1)-'DRC-BDRC'!W2)&gt;0,(TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!W1)-'DRC-BDRC'!W2),0))</f>
+        <v>0</v>
       </c>
       <c r="X2" s="3" cm="1">
-        <f t="array" ref="X2">_xlfn.SINGLE(IF((TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!X1)-'DRC-BDRC'!X2)&gt;0,(TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!X1)-'DRC-BDRC'!X2),0))</f>
-        <v>224.80061291150741</v>
+        <f t="array" ref="X2">_xlfn.SINGLE(IF((TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!X1)-'DRC-BDRC'!X2)&gt;0,(TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!X1)-'DRC-BDRC'!X2),0))</f>
+        <v>0</v>
       </c>
       <c r="Y2" s="3" cm="1">
-        <f t="array" ref="Y2">_xlfn.SINGLE(IF((TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!Y1)-'DRC-BDRC'!Y2)&gt;0,(TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!Y1)-'DRC-BDRC'!Y2),0))</f>
-        <v>271.31807421165286</v>
+        <f t="array" ref="Y2">_xlfn.SINGLE(IF((TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!Y1)-'DRC-BDRC'!Y2)&gt;0,(TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!Y1)-'DRC-BDRC'!Y2),0))</f>
+        <v>0</v>
       </c>
       <c r="Z2" s="3" cm="1">
-        <f t="array" ref="Z2">_xlfn.SINGLE(IF((TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!Z1)-'DRC-BDRC'!Z2)&gt;0,(TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!Z1)-'DRC-BDRC'!Z2),0))</f>
-        <v>315.10055247958644</v>
+        <f t="array" ref="Z2">_xlfn.SINGLE(IF((TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!Z1)-'DRC-BDRC'!Z2)&gt;0,(TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!Z1)-'DRC-BDRC'!Z2),0))</f>
+        <v>0</v>
       </c>
       <c r="AA2" s="3" cm="1">
-        <f t="array" ref="AA2">_xlfn.SINGLE(IF((TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!AA1)-'DRC-BDRC'!AA2)&gt;0,(TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!AA1)-'DRC-BDRC'!AA2),0))</f>
-        <v>356.08763316474688</v>
+        <f t="array" ref="AA2">_xlfn.SINGLE(IF((TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!AA1)-'DRC-BDRC'!AA2)&gt;0,(TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!AA1)-'DRC-BDRC'!AA2),0))</f>
+        <v>0</v>
       </c>
       <c r="AB2" s="3" cm="1">
-        <f t="array" ref="AB2">_xlfn.SINGLE(IF((TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!AB1)-'DRC-BDRC'!AB2)&gt;0,(TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!AB1)-'DRC-BDRC'!AB2),0))</f>
-        <v>394.21756718620054</v>
+        <f t="array" ref="AB2">_xlfn.SINGLE(IF((TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!AB1)-'DRC-BDRC'!AB2)&gt;0,(TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!AB1)-'DRC-BDRC'!AB2),0))</f>
+        <v>0</v>
       </c>
       <c r="AC2" s="3" cm="1">
-        <f t="array" ref="AC2">_xlfn.SINGLE(IF((TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!AC1)-'DRC-BDRC'!AC2)&gt;0,(TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!AC1)-'DRC-BDRC'!AC2),0))</f>
-        <v>429.42724145346619</v>
+        <f t="array" ref="AC2">_xlfn.SINGLE(IF((TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!AC1)-'DRC-BDRC'!AC2)&gt;0,(TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!AC1)-'DRC-BDRC'!AC2),0))</f>
+        <v>0</v>
       </c>
       <c r="AD2" s="3" cm="1">
-        <f t="array" ref="AD2">_xlfn.SINGLE(IF((TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!AD1)-'DRC-BDRC'!AD2)&gt;0,(TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!AD1)-'DRC-BDRC'!AD2),0))</f>
-        <v>461.6521487360942</v>
+        <f t="array" ref="AD2">_xlfn.SINGLE(IF((TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!AD1)-'DRC-BDRC'!AD2)&gt;0,(TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!AD1)-'DRC-BDRC'!AD2),0))</f>
+        <v>0</v>
       </c>
       <c r="AE2" s="3" cm="1">
-        <f t="array" ref="AE2">_xlfn.SINGLE(IF((TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!AE1)-'DRC-BDRC'!AE2)&gt;0,(TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!AE1)-'DRC-BDRC'!AE2),0))</f>
-        <v>490.82635686797494</v>
+        <f t="array" ref="AE2">_xlfn.SINGLE(IF((TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!AE1)-'DRC-BDRC'!AE2)&gt;0,(TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!AE1)-'DRC-BDRC'!AE2),0))</f>
+        <v>0</v>
       </c>
       <c r="AF2" s="3" cm="1">
-        <f t="array" ref="AF2">_xlfn.SINGLE(IF((TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!AF1)-'DRC-BDRC'!AF2)&gt;0,(TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!AF1)-'DRC-BDRC'!AF2),0))</f>
-        <v>516.88247727079306</v>
+        <f t="array" ref="AF2">_xlfn.SINGLE(IF((TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!AF1)-'DRC-BDRC'!AF2)&gt;0,(TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!AF1)-'DRC-BDRC'!AF2),0))</f>
+        <v>0</v>
       </c>
       <c r="AG2" s="3" cm="1">
-        <f t="array" ref="AG2">_xlfn.SINGLE(IF((TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!AG1)-'DRC-BDRC'!AG2)&gt;0,(TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!AG1)-'DRC-BDRC'!AG2),0))</f>
-        <v>539.7516327827725</v>
+        <f t="array" ref="AG2">_xlfn.SINGLE(IF((TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!AG1)-'DRC-BDRC'!AG2)&gt;0,(TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!AG1)-'DRC-BDRC'!AG2),0))</f>
+        <v>0</v>
       </c>
       <c r="AH2" s="3" cm="1">
-        <f t="array" ref="AH2">_xlfn.SINGLE(IF((TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!AH1)-'DRC-BDRC'!AH2)&gt;0,(TREND(MOTIE!$E$5:$T$5,MOTIE!$E$4:$T$4,'DRC-PADRC'!AH1)-'DRC-BDRC'!AH2),0))</f>
-        <v>559.36342477647395</v>
+        <f t="array" ref="AH2">_xlfn.SINGLE(IF((TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!AH1)-'DRC-BDRC'!AH2)&gt;0,(TREND(MOTIE!$H$5:$V$5,MOTIE!$H$4:$V$4,'DRC-PADRC'!AH1)-'DRC-BDRC'!AH2),0))</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1788,22 +1849,22 @@
     <tabColor rgb="FF002060"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="21.3984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A1" s="26" t="s">
-        <v>25</v>
-      </c>
-      <c r="B1" s="27" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:2">
+      <c r="A1" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="23" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="B2" s="3">
         <f>ROUND(MOTIE!A20,0)</f>
@@ -1817,9 +1878,9 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E59C87379D9A4242BB3A95F198D6F941" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="07a235b40ffe2d9a960bde50f6511605">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="40f4d404-d193-41dc-bb72-733c1e774208" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="485fc8e6f691b86ce0aee9b7e82feca0" ns2:_="">
-    <xsd:import namespace="40f4d404-d193-41dc-bb72-733c1e774208"/>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="문서" ma:contentTypeID="0x01010027350D42B0D95040ACC873ED5DCB146E" ma:contentTypeVersion="10" ma:contentTypeDescription="새 문서를 만듭니다." ma:contentTypeScope="" ma:versionID="c2e4f52adf7af47ba555973ff8cbcabe">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="688c5d3b-a76a-458b-b159-91c2a1154680" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="502e33886199ad3dabc1cc93359c84e5" ns2:_="">
+    <xsd:import namespace="688c5d3b-a76a-458b-b159-91c2a1154680"/>
     <xsd:element name="properties">
       <xsd:complexType>
         <xsd:sequence>
@@ -1830,6 +1891,11 @@
                 <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -1837,7 +1903,7 @@
       </xsd:complexType>
     </xsd:element>
   </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="40f4d404-d193-41dc-bb72-733c1e774208" elementFormDefault="qualified">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="688c5d3b-a76a-458b-b159-91c2a1154680" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
@@ -1860,6 +1926,33 @@
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="12" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="13" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="14" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="15" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="17" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="이미지 태그" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="eca5b831-c3dc-41cf-bd85-218b82cecb21" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
   </xsd:schema>
   <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
     <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
@@ -1870,8 +1963,8 @@
         <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="콘텐츠 형식"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="제목"/>
         <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
         <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
@@ -1961,6 +2054,16 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="688c5d3b-a76a-458b-b159-91c2a1154680">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -1969,20 +2072,44 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2411B9C5-6668-4E56-BAD3-E55E88156D50}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5A435F18-B230-45AD-9E6F-1D5E2C9E6E8C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="688c5d3b-a76a-458b-b159-91c2a1154680"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{122FCCFF-E84B-4F37-AF43-02E257308C42}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{19650D19-B906-4A4F-BC60-F0340A4F044A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="688c5d3b-a76a-458b-b159-91c2a1154680"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{19650D19-B906-4A4F-BC60-F0340A4F044A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{122FCCFF-E84B-4F37-AF43-02E257308C42}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{c7ef1c8b-ba63-4702-8e74-5094387a97de}" enabled="0" method="" siteId="{c7ef1c8b-ba63-4702-8e74-5094387a97de}" removed="1"/>
+</clbl:labelList>
 </file>
</xml_diff>